<commit_message>
Migra datos de Elche a data raw
</commit_message>
<xml_diff>
--- a/outputs/document_embeddings_muestra.xlsx
+++ b/outputs/document_embeddings_muestra.xlsx
@@ -486,7 +486,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>doc_0334</t>
+          <t>doc_0201</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -511,7 +511,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>documentos_ceei_elche_PDF/Informes_y_Publicaciones/Informe COTEC 2014.pdf</t>
+          <t>data/raw/ceei_elche/pdf/Informes_y_Publicaciones/Informe COTEC 2014.pdf</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
@@ -545,7 +545,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>doc_0344</t>
+          <t>doc_0211</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -570,7 +570,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>documentos_ceei_elche_PDF/Informes_y_Publicaciones/Informe GEM 2018-19 sobre el ecosistema emprendedor en España.pdf</t>
+          <t>data/raw/ceei_elche/pdf/Informes_y_Publicaciones/Informe GEM 2018-19 sobre el ecosistema emprendedor en España.pdf</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
@@ -604,7 +604,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>doc_0323</t>
+          <t>doc_0190</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -629,7 +629,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>documentos_ceei_elche_PDF/Informes_y_Publicaciones/Análisis para la definición de las competencias del perfil profesional de un Agente de Desarrollo Local_.pdf</t>
+          <t>data/raw/ceei_elche/pdf/Informes_y_Publicaciones/Análisis para la definición de las competencias del perfil profesional de un Agente de Desarrollo Local_.pdf</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
@@ -663,7 +663,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>doc_0327</t>
+          <t>doc_0194</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -688,7 +688,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>documentos_ceei_elche_PDF/Informes_y_Publicaciones/Estudio integral sobre el sector marítimo_recreativo en la Comunidad Valenciana.pdf</t>
+          <t>data/raw/ceei_elche/pdf/Informes_y_Publicaciones/Estudio integral sobre el sector marítimo_recreativo en la Comunidad Valenciana.pdf</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
@@ -722,7 +722,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>doc_0337</t>
+          <t>doc_0204</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -747,7 +747,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>documentos_ceei_elche_PDF/Informes_y_Publicaciones/Informe de resultados 2023_ HUB Nueva Ruralidad RegenerativaLo rural como punta de lanza de la transformación económica_.pdf</t>
+          <t>data/raw/ceei_elche/pdf/Informes_y_Publicaciones/Informe de resultados 2023_ HUB Nueva Ruralidad RegenerativaLo rural como punta de lanza de la transformación económica_.pdf</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
@@ -781,7 +781,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>doc_0328</t>
+          <t>doc_0195</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -806,7 +806,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>documentos_ceei_elche_PDF/Informes_y_Publicaciones/Estudio sobre creación de un Fondo de Garantía para la concesión de microcréditosInformes y estudios.pdf</t>
+          <t>data/raw/ceei_elche/pdf/Informes_y_Publicaciones/Estudio sobre creación de un Fondo de Garantía para la concesión de microcréditosInformes y estudios.pdf</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
@@ -840,7 +840,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>doc_0347</t>
+          <t>doc_0214</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -865,7 +865,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>documentos_ceei_elche_PDF/Informes_y_Publicaciones/Resultados proyecto piloto HUB Innovación Colaborativa Territorial 2021 - 2022.pdf</t>
+          <t>data/raw/ceei_elche/pdf/Informes_y_Publicaciones/Resultados proyecto piloto HUB Innovación Colaborativa Territorial 2021 - 2022.pdf</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
@@ -899,7 +899,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>doc_0332</t>
+          <t>doc_0199</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -924,7 +924,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>documentos_ceei_elche_PDF/Informes_y_Publicaciones/Informe Benchmarking CEEI Elche 2018-2019_ Análisis sobre metodologías y herramientas de innovación_Informes y estudios.pdf</t>
+          <t>data/raw/ceei_elche/pdf/Informes_y_Publicaciones/Informe Benchmarking CEEI Elche 2018-2019_ Análisis sobre metodologías y herramientas de innovación_Informes y estudios.pdf</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
@@ -958,7 +958,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>doc_0324</t>
+          <t>doc_0191</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -983,7 +983,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>documentos_ceei_elche_PDF/Informes_y_Publicaciones/Análisis sobre metodologías y herramientas de innovación del ecosistema emprendedor de CVInformes y estudios.pdf</t>
+          <t>data/raw/ceei_elche/pdf/Informes_y_Publicaciones/Análisis sobre metodologías y herramientas de innovación del ecosistema emprendedor de CVInformes y estudios.pdf</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
@@ -1017,7 +1017,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>doc_0322</t>
+          <t>doc_0189</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1042,7 +1042,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>documentos_ceei_elche_PDF/Informes_y_Publicaciones/Análisis de la capacidad tractora de las empresas de la Provincia de AlicanteIdentificación de las micro y pequeñas empr.pdf</t>
+          <t>data/raw/ceei_elche/pdf/Informes_y_Publicaciones/Análisis de la capacidad tractora de las empresas de la Provincia de AlicanteIdentificación de las micro y pequeñas empr.pdf</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>

</xml_diff>